<commit_message>
chore(demo): nombres descriptivos sin siglas (MDS->Maxima densidad seca, OCH->Humedad optima)
</commit_message>
<xml_diff>
--- a/Actividadesv1/CAD_ConoArena_Demo.xlsx
+++ b/Actividadesv1/CAD_ConoArena_Demo.xlsx
@@ -830,7 +830,7 @@
         <v>21</v>
       </c>
       <c r="D22" t="str">
-        <v>Máxima densidad seca MDS — Proctor (g/cm³)</v>
+        <v>Máxima densidad seca del Proctor (g/cm³)</v>
       </c>
       <c r="E22" t="str">
         <v>xref-[#20A].19A</v>
@@ -850,7 +850,7 @@
         <v>22</v>
       </c>
       <c r="D23" t="str">
-        <v>Óptimo contenido de humedad OCH — Proctor (%)</v>
+        <v>Humedad óptima del Proctor (%)</v>
       </c>
       <c r="E23" t="str">
         <v>xref-[#20A].20A</v>

</xml_diff>